<commit_message>
Module 1: rebuild Rook company docs — no agencies, seven-person roster, seams relocated
</commit_message>
<xml_diff>
--- a/00-rook/company/who-does-what.xlsx
+++ b/00-rook/company/who-does-what.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Team" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -475,7 +475,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Product, Engineering, Support and Partnerships · last updated 2 September 2026</t>
+          <t>Product, Engineering, Design, Support and Data · last updated 2 September 2026</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Roadmap, quarterly commitments, partner escalations</t>
+          <t>Roadmap and commitments</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -574,22 +574,22 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Grant Whitlow</t>
+          <t>Marcus Oyelaran</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Product Manager</t>
+          <t>Engineering Manager</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>Supply</t>
+          <t>Dispatch</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Requisitions, maintenance scheduling, field failure reports</t>
+          <t>The Dispatch engineering team</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -602,12 +602,12 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Marcus Oyelaran</t>
+          <t>Wen Li</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Engineering Manager</t>
+          <t>Staff Engineer</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -617,25 +617,29 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Dispatch engineering team</t>
+          <t>Built the part that decides who gets pinged</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>Chicago</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr"/>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Away 14–24 Aug 2026</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Wen Li</t>
+          <t>Sofia Marino</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Staff Engineer</t>
+          <t>Product Designer</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -645,39 +649,35 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Callout routing service</t>
+          <t>Console and phone app</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>Berlin</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Built the routing service</t>
-        </is>
-      </c>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Tomás Ferreira</t>
+          <t>Nadia Hoffmann</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer</t>
+          <t>Support Lead</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Dispatch</t>
+          <t>Dispatch &amp; Supply</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Responder mobile app</t>
+          <t>The tickets</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -690,204 +690,32 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Aisha Nkemelu</t>
+          <t>Ravi Menon</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Software Engineer</t>
+          <t>Data Analyst</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Dispatch</t>
+          <t>Dispatch &amp; Supply</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Dispatch API and console back end</t>
+          <t>The numbers. Reports weekly on how often responders are answering.</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Chicago</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Sofia Marino</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Product Designer</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Dispatch</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Console and mobile design</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>Chicago</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Nadia Hoffmann</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Support Lead</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Dispatch &amp; Supply</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>Ticket triage and escalation</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>Berlin</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Jonas Brandt</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Customer Success Manager</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Dispatch &amp; Supply</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>Mid-market agency accounts</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>Berlin</t>
-        </is>
-      </c>
-      <c r="F14" s="5" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>Beatrix Sandoval</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Head of Agency Partnerships</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Dispatch &amp; Supply</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>Enterprise accounts, including Meridian Protective Group</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>Chicago</t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Ravi Menon</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Data Analyst</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>Dispatch &amp; Supply</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>Metrics, dashboards, weekly acceptance reporting</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="inlineStr">
-        <is>
           <t>Singapore</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>Shared across both surfaces; requests go through #data</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Iris Kowalczyk</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>QA Lead</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>Dispatch</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>Release verification</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>Berlin</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>On leave through 25 Sept 2026</t>
         </is>
       </c>
     </row>

</xml_diff>